<commit_message>
Remove dataset upload, my-uploads, and download APK modules, remove backend upload APIs, and update README
</commit_message>
<xml_diff>
--- a/Test_Execution_Report.xlsx
+++ b/Test_Execution_Report.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All Test Results" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Appium Mobile Suite" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Selenium Web Suite" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Load Test Analysis" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Test Results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appium Mobile Suite" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selenium Web Suite" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Load Test Analysis" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -531,7 +531,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-08 17:13:05</t>
+          <t>2026-10-11 14:04:56</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>1906.0 req/sec</t>
+          <t>15.07 req/sec</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>181.55 ms</t>
+          <t>800.07 ms</t>
         </is>
       </c>
     </row>
@@ -2912,17 +2912,17 @@
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>Web UI Form</t>
+          <t>Web Citation</t>
         </is>
       </c>
       <c r="E64" s="10" t="inlineStr">
         <is>
-          <t>Upload CSV Gene Association File</t>
+          <t>Generate BibTeX Citation for Disease Record</t>
         </is>
       </c>
       <c r="F64" s="10" t="n">
@@ -2948,17 +2948,17 @@
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>Web UI Form</t>
+          <t>Web Citation</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>Upload TSV Pathway Annotation File</t>
+          <t>Generate RIS Citation for Gene Record</t>
         </is>
       </c>
       <c r="F65" s="12" t="n">
@@ -2984,17 +2984,17 @@
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>Web UI Form</t>
+          <t>Web Citation</t>
         </is>
       </c>
       <c r="E66" s="10" t="inlineStr">
         <is>
-          <t>Upload VCF Variant Calling File</t>
+          <t>Generate APA Citation for Association Record</t>
         </is>
       </c>
       <c r="F66" s="10" t="n">
@@ -3020,17 +3020,17 @@
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>Web UI Validation</t>
+          <t>Web Export</t>
         </is>
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>Upload File Size Limit (Max 50MB) Enforcement</t>
+          <t>Download Search Results as Formatted CSV</t>
         </is>
       </c>
       <c r="F67" s="12" t="n">
@@ -3056,17 +3056,17 @@
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>Security Check</t>
+          <t>Web Export</t>
         </is>
       </c>
       <c r="E68" s="10" t="inlineStr">
         <is>
-          <t>Invalid File Extension Upload Rejection (.exe/.sh)</t>
+          <t>Download Search Results as Structured JSON</t>
         </is>
       </c>
       <c r="F68" s="10" t="n">
@@ -3092,17 +3092,17 @@
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
-          <t>Web UI Parsing</t>
+          <t>Web Export</t>
         </is>
       </c>
       <c r="E69" s="12" t="inlineStr">
         <is>
-          <t>Malformed CSV Header Validation Error display</t>
+          <t>Export Association Matrix as Excel File</t>
         </is>
       </c>
       <c r="F69" s="12" t="n">
@@ -3128,17 +3128,17 @@
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>Web UI Table</t>
+          <t>Web Interactive</t>
         </is>
       </c>
       <c r="E70" s="10" t="inlineStr">
         <is>
-          <t>View User Dataset Upload History List</t>
+          <t>Copy Citation String to System Clipboard</t>
         </is>
       </c>
       <c r="F70" s="10" t="n">
@@ -3164,17 +3164,17 @@
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>Web Download</t>
+          <t>Web Data</t>
         </is>
       </c>
       <c r="E71" s="12" t="inlineStr">
         <is>
-          <t>Download Previously Uploaded User File</t>
+          <t>Verify Citation Year and DOID / Ensembl Metadata</t>
         </is>
       </c>
       <c r="F71" s="12" t="n">
@@ -3200,17 +3200,17 @@
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>Web UI Action</t>
+          <t>Web Export</t>
         </is>
       </c>
       <c r="E72" s="10" t="inlineStr">
         <is>
-          <t>Delete Uploaded Dataset Record</t>
+          <t>Export Filtered Query Results with Active Facets</t>
         </is>
       </c>
       <c r="F72" s="10" t="n">
@@ -3236,17 +3236,17 @@
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>Web UI Async</t>
+          <t>Web Standard</t>
         </is>
       </c>
       <c r="E73" s="12" t="inlineStr">
         <is>
-          <t>Ingestion Progress Bar Web Socket / Polling</t>
+          <t>Data Export File Character Encoding (UTF-8)</t>
         </is>
       </c>
       <c r="F73" s="12" t="n">
@@ -6238,7 +6238,7 @@
         </is>
       </c>
       <c r="F156" s="10" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="G156" s="11" t="inlineStr">
         <is>
@@ -6332,17 +6332,17 @@
       </c>
       <c r="C159" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D159" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Chooser</t>
+          <t>Mobile Storage</t>
         </is>
       </c>
       <c r="E159" s="12" t="inlineStr">
         <is>
-          <t>Tap Pick File Button to Launch Android Storage Intent</t>
+          <t>Add Disease to Mobile Local Favorites Storage</t>
         </is>
       </c>
       <c r="F159" s="12" t="n">
@@ -6368,7 +6368,7 @@
       </c>
       <c r="C160" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D160" s="10" t="inlineStr">
@@ -6378,7 +6378,7 @@
       </c>
       <c r="E160" s="10" t="inlineStr">
         <is>
-          <t>Select CSV Dataset File from Mobile Download Folder</t>
+          <t>Add Gene to Mobile Local Favorites Storage</t>
         </is>
       </c>
       <c r="F160" s="10" t="n">
@@ -6404,17 +6404,17 @@
       </c>
       <c r="C161" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D161" s="12" t="inlineStr">
         <is>
-          <t>Mobile Hardware</t>
+          <t>Mobile UI</t>
         </is>
       </c>
       <c r="E161" s="12" t="inlineStr">
         <is>
-          <t>Use Device Camera to Scan Dataset QR / Barcode Link</t>
+          <t>View Saved Lists Tab with Filtered Records</t>
         </is>
       </c>
       <c r="F161" s="12" t="n">
@@ -6440,17 +6440,17 @@
       </c>
       <c r="C162" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D162" s="10" t="inlineStr">
         <is>
-          <t>Mobile UI</t>
+          <t>Mobile Interactive</t>
         </is>
       </c>
       <c r="E162" s="10" t="inlineStr">
         <is>
-          <t>Mobile Upload Progress Bar &amp; Percentage Meter</t>
+          <t>Remove Saved Item via Unbookmark Button</t>
         </is>
       </c>
       <c r="F162" s="10" t="n">
@@ -6476,17 +6476,17 @@
       </c>
       <c r="C163" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D163" s="12" t="inlineStr">
         <is>
-          <t>Mobile Action</t>
+          <t>Mobile Storage</t>
         </is>
       </c>
       <c r="E163" s="12" t="inlineStr">
         <is>
-          <t>Cancel Upload Button Tap Interruption Check</t>
+          <t>Persist Recent Searches in Mobile localStorage</t>
         </is>
       </c>
       <c r="F163" s="12" t="n">
@@ -6512,17 +6512,17 @@
       </c>
       <c r="C164" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D164" s="10" t="inlineStr">
         <is>
-          <t>Mobile Security</t>
+          <t>Mobile Action</t>
         </is>
       </c>
       <c r="E164" s="10" t="inlineStr">
         <is>
-          <t>Mobile Storage READ/WRITE Permission Alert Request</t>
+          <t>Clear All Mobile Recent Search History Cards</t>
         </is>
       </c>
       <c r="F164" s="10" t="n">
@@ -6548,17 +6548,17 @@
       </c>
       <c r="C165" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D165" s="12" t="inlineStr">
         <is>
-          <t>Mobile Validation</t>
+          <t>Mobile System</t>
         </is>
       </c>
       <c r="E165" s="12" t="inlineStr">
         <is>
-          <t>Invalid File Extension Mobile Toast Error Alert</t>
+          <t>Copy Record Citation Text to Android Clipboard</t>
         </is>
       </c>
       <c r="F165" s="12" t="n">
@@ -6584,17 +6584,17 @@
       </c>
       <c r="C166" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D166" s="10" t="inlineStr">
         <is>
-          <t>Mobile UI</t>
+          <t>Mobile Export</t>
         </is>
       </c>
       <c r="E166" s="10" t="inlineStr">
         <is>
-          <t>Preview Uploaded Dataset Columns in Mobile Table View</t>
+          <t>Export Bookmarked List as JSON / Text</t>
         </is>
       </c>
       <c r="F166" s="10" t="n">
@@ -6620,17 +6620,17 @@
       </c>
       <c r="C167" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D167" s="12" t="inlineStr">
         <is>
-          <t>Mobile Action</t>
+          <t>Mobile UI Badge</t>
         </is>
       </c>
       <c r="E167" s="12" t="inlineStr">
         <is>
-          <t>Delete Uploaded Dataset via Mobile Swipe Action</t>
+          <t>Display Active Saved Count Badge on Bottom Nav</t>
         </is>
       </c>
       <c r="F167" s="12" t="n">
@@ -6656,17 +6656,17 @@
       </c>
       <c r="C168" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D168" s="10" t="inlineStr">
         <is>
-          <t>Mobile Notification</t>
+          <t>Mobile Offline</t>
         </is>
       </c>
       <c r="E168" s="10" t="inlineStr">
         <is>
-          <t>Background Ingestion Android Notification Banner Trigger</t>
+          <t>Offline Local Cache Retrieval on Network Disconnect</t>
         </is>
       </c>
       <c r="F168" s="10" t="n">
@@ -9915,7 +9915,7 @@
         </is>
       </c>
       <c r="F56" s="10" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
@@ -10009,17 +10009,17 @@
       </c>
       <c r="C59" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Chooser</t>
+          <t>Mobile Storage</t>
         </is>
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>Tap Pick File Button to Launch Android Storage Intent</t>
+          <t>Add Disease to Mobile Local Favorites Storage</t>
         </is>
       </c>
       <c r="F59" s="12" t="n">
@@ -10045,7 +10045,7 @@
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
@@ -10055,7 +10055,7 @@
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>Select CSV Dataset File from Mobile Download Folder</t>
+          <t>Add Gene to Mobile Local Favorites Storage</t>
         </is>
       </c>
       <c r="F60" s="10" t="n">
@@ -10081,17 +10081,17 @@
       </c>
       <c r="C61" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D61" s="12" t="inlineStr">
         <is>
-          <t>Mobile Hardware</t>
+          <t>Mobile UI</t>
         </is>
       </c>
       <c r="E61" s="12" t="inlineStr">
         <is>
-          <t>Use Device Camera to Scan Dataset QR / Barcode Link</t>
+          <t>View Saved Lists Tab with Filtered Records</t>
         </is>
       </c>
       <c r="F61" s="12" t="n">
@@ -10117,17 +10117,17 @@
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>Mobile UI</t>
+          <t>Mobile Interactive</t>
         </is>
       </c>
       <c r="E62" s="10" t="inlineStr">
         <is>
-          <t>Mobile Upload Progress Bar &amp; Percentage Meter</t>
+          <t>Remove Saved Item via Unbookmark Button</t>
         </is>
       </c>
       <c r="F62" s="10" t="n">
@@ -10153,17 +10153,17 @@
       </c>
       <c r="C63" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D63" s="12" t="inlineStr">
         <is>
-          <t>Mobile Action</t>
+          <t>Mobile Storage</t>
         </is>
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
-          <t>Cancel Upload Button Tap Interruption Check</t>
+          <t>Persist Recent Searches in Mobile localStorage</t>
         </is>
       </c>
       <c r="F63" s="12" t="n">
@@ -10189,17 +10189,17 @@
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>Mobile Security</t>
+          <t>Mobile Action</t>
         </is>
       </c>
       <c r="E64" s="10" t="inlineStr">
         <is>
-          <t>Mobile Storage READ/WRITE Permission Alert Request</t>
+          <t>Clear All Mobile Recent Search History Cards</t>
         </is>
       </c>
       <c r="F64" s="10" t="n">
@@ -10225,17 +10225,17 @@
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>Mobile Validation</t>
+          <t>Mobile System</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>Invalid File Extension Mobile Toast Error Alert</t>
+          <t>Copy Record Citation Text to Android Clipboard</t>
         </is>
       </c>
       <c r="F65" s="12" t="n">
@@ -10261,17 +10261,17 @@
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>Mobile UI</t>
+          <t>Mobile Export</t>
         </is>
       </c>
       <c r="E66" s="10" t="inlineStr">
         <is>
-          <t>Preview Uploaded Dataset Columns in Mobile Table View</t>
+          <t>Export Bookmarked List as JSON / Text</t>
         </is>
       </c>
       <c r="F66" s="10" t="n">
@@ -10297,17 +10297,17 @@
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>Mobile Action</t>
+          <t>Mobile UI Badge</t>
         </is>
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>Delete Uploaded Dataset via Mobile Swipe Action</t>
+          <t>Display Active Saved Count Badge on Bottom Nav</t>
         </is>
       </c>
       <c r="F67" s="12" t="n">
@@ -10333,17 +10333,17 @@
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>Mobile File Upload</t>
+          <t>Mobile Favorites</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>Mobile Notification</t>
+          <t>Mobile Offline</t>
         </is>
       </c>
       <c r="E68" s="10" t="inlineStr">
         <is>
-          <t>Background Ingestion Android Notification Banner Trigger</t>
+          <t>Offline Local Cache Retrieval on Network Disconnect</t>
         </is>
       </c>
       <c r="F68" s="10" t="n">
@@ -13866,17 +13866,17 @@
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>Web UI Form</t>
+          <t>Web Citation</t>
         </is>
       </c>
       <c r="E64" s="10" t="inlineStr">
         <is>
-          <t>Upload CSV Gene Association File</t>
+          <t>Generate BibTeX Citation for Disease Record</t>
         </is>
       </c>
       <c r="F64" s="10" t="n">
@@ -13902,17 +13902,17 @@
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>Web UI Form</t>
+          <t>Web Citation</t>
         </is>
       </c>
       <c r="E65" s="12" t="inlineStr">
         <is>
-          <t>Upload TSV Pathway Annotation File</t>
+          <t>Generate RIS Citation for Gene Record</t>
         </is>
       </c>
       <c r="F65" s="12" t="n">
@@ -13938,17 +13938,17 @@
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>Web UI Form</t>
+          <t>Web Citation</t>
         </is>
       </c>
       <c r="E66" s="10" t="inlineStr">
         <is>
-          <t>Upload VCF Variant Calling File</t>
+          <t>Generate APA Citation for Association Record</t>
         </is>
       </c>
       <c r="F66" s="10" t="n">
@@ -13974,17 +13974,17 @@
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>Web UI Validation</t>
+          <t>Web Export</t>
         </is>
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>Upload File Size Limit (Max 50MB) Enforcement</t>
+          <t>Download Search Results as Formatted CSV</t>
         </is>
       </c>
       <c r="F67" s="12" t="n">
@@ -14010,17 +14010,17 @@
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>Security Check</t>
+          <t>Web Export</t>
         </is>
       </c>
       <c r="E68" s="10" t="inlineStr">
         <is>
-          <t>Invalid File Extension Upload Rejection (.exe/.sh)</t>
+          <t>Download Search Results as Structured JSON</t>
         </is>
       </c>
       <c r="F68" s="10" t="n">
@@ -14046,17 +14046,17 @@
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
-          <t>Web UI Parsing</t>
+          <t>Web Export</t>
         </is>
       </c>
       <c r="E69" s="12" t="inlineStr">
         <is>
-          <t>Malformed CSV Header Validation Error display</t>
+          <t>Export Association Matrix as Excel File</t>
         </is>
       </c>
       <c r="F69" s="12" t="n">
@@ -14082,17 +14082,17 @@
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>Web UI Table</t>
+          <t>Web Interactive</t>
         </is>
       </c>
       <c r="E70" s="10" t="inlineStr">
         <is>
-          <t>View User Dataset Upload History List</t>
+          <t>Copy Citation String to System Clipboard</t>
         </is>
       </c>
       <c r="F70" s="10" t="n">
@@ -14118,17 +14118,17 @@
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>Web Download</t>
+          <t>Web Data</t>
         </is>
       </c>
       <c r="E71" s="12" t="inlineStr">
         <is>
-          <t>Download Previously Uploaded User File</t>
+          <t>Verify Citation Year and DOID / Ensembl Metadata</t>
         </is>
       </c>
       <c r="F71" s="12" t="n">
@@ -14154,17 +14154,17 @@
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>Web UI Action</t>
+          <t>Web Export</t>
         </is>
       </c>
       <c r="E72" s="10" t="inlineStr">
         <is>
-          <t>Delete Uploaded Dataset Record</t>
+          <t>Export Filtered Query Results with Active Facets</t>
         </is>
       </c>
       <c r="F72" s="10" t="n">
@@ -14190,17 +14190,17 @@
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>File Upload</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
         <is>
-          <t>Web UI Async</t>
+          <t>Web Standard</t>
         </is>
       </c>
       <c r="E73" s="12" t="inlineStr">
         <is>
-          <t>Ingestion Progress Bar Web Socket / Polling</t>
+          <t>Data Export File Character Encoding (UTF-8)</t>
         </is>
       </c>
       <c r="F73" s="12" t="n">
@@ -15377,7 +15377,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>10.2 Seconds</t>
+          <t>15.26 Seconds</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>19448 Reqs</t>
+          <t>230 Reqs</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
@@ -15421,7 +15421,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>1906.0 req/sec</t>
+          <t>15.07 req/sec</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
@@ -15443,7 +15443,7 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>181.55 ms</t>
+          <t>800.07 ms</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>45.01 ms</t>
+          <t>45.21 ms</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -15487,7 +15487,7 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>320.0 ms</t>
+          <t>7574.21 ms</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -15509,7 +15509,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>305.81 ms</t>
+          <t>5180.39 ms</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -15531,7 +15531,7 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>0.0 %</t>
+          <t>6.52 %</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Add full 100 Appium and 100 Selenium test suites, 1-min baseline load testing, and unified Excel analysis report
</commit_message>
<xml_diff>
--- a/Test_Execution_Report.xlsx
+++ b/Test_Execution_Report.xlsx
@@ -531,7 +531,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-11 14:04:56</t>
+          <t>2026-10-28 17:11:43</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>15.07 req/sec</t>
+          <t>20.22 req/sec</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>800.07 ms</t>
+          <t>256.75 ms</t>
         </is>
       </c>
     </row>
@@ -15377,7 +15377,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>15.26 Seconds</t>
+          <t>64.99 Seconds</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>230 Reqs</t>
+          <t>1314 Reqs</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
@@ -15421,7 +15421,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>15.07 req/sec</t>
+          <t>20.22 req/sec</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
@@ -15443,7 +15443,7 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>800.07 ms</t>
+          <t>256.75 ms</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>45.21 ms</t>
+          <t>50.03 ms</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -15487,7 +15487,7 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>7574.21 ms</t>
+          <t>1475.25 ms</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -15509,7 +15509,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>5180.39 ms</t>
+          <t>633.67 ms</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -15531,7 +15531,7 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>6.52 %</t>
+          <t>0.0 %</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">

</xml_diff>